<commit_message>
Refactor code mappings for CE, CS, and CD 5c2416fdf341467b5b13bb953b62476f183326c0
</commit_message>
<xml_diff>
--- a/fsh/ig/CdaToCodeConceptMap.xlsx
+++ b/fsh/ig/CdaToCodeConceptMap.xlsx
@@ -65,7 +65,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-13T09:48:02+00:00</t>
+    <t>2026-04-13T09:58:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -122,28 +122,28 @@
     <t>CE.code</t>
   </si>
   <si>
+    <t>equivalent</t>
+  </si>
+  <si>
+    <t>code</t>
+  </si>
+  <si>
+    <t>http://hl7.org/fhir/StructureDefinition/CodeableConcept</t>
+  </si>
+  <si>
+    <t>CE.originalText</t>
+  </si>
+  <si>
+    <t>CodeableConcept.text</t>
+  </si>
+  <si>
+    <t>CodeableConcept.coding.code</t>
+  </si>
+  <si>
+    <t>CE.codeSystem</t>
+  </si>
+  <si>
     <t>related-to</t>
-  </si>
-  <si>
-    <t>code.value</t>
-  </si>
-  <si>
-    <t>http://hl7.org/fhir/StructureDefinition/CodeableConcept</t>
-  </si>
-  <si>
-    <t>CE.originalText</t>
-  </si>
-  <si>
-    <t>equivalent</t>
-  </si>
-  <si>
-    <t>CodeableConcept.text</t>
-  </si>
-  <si>
-    <t>CodeableConcept.coding.code</t>
-  </si>
-  <si>
-    <t>CE.codeSystem</t>
   </si>
   <si>
     <t>CodeableConcept.coding.system</t>
@@ -547,13 +547,13 @@
         <v>37</v>
       </c>
       <c r="C3" t="s" s="2">
+        <v>34</v>
+      </c>
+      <c r="D3" t="s" s="2">
         <v>38</v>
       </c>
-      <c r="D3" t="s" s="2">
-        <v>39</v>
-      </c>
       <c r="E3" t="s" s="2">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
@@ -564,24 +564,24 @@
         <v>33</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="B5" t="s" s="2">
+        <v>40</v>
+      </c>
+      <c r="C5" t="s" s="2">
         <v>41</v>
-      </c>
-      <c r="B5" t="s" s="2">
-        <v>41</v>
-      </c>
-      <c r="C5" t="s" s="2">
-        <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
         <v>42</v>
@@ -598,7 +598,7 @@
         <v>43</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
         <v>44</v>
@@ -615,7 +615,7 @@
         <v>45</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s" s="2">
         <v>46</v>
@@ -676,7 +676,7 @@
         <v>49</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
         <v>35</v>
@@ -737,13 +737,13 @@
         <v>49</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -798,7 +798,7 @@
         <v>51</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s" s="2">
         <v>35</v>
@@ -859,13 +859,13 @@
         <v>52</v>
       </c>
       <c r="C3" t="s" s="2">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E3" t="s" s="2">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4">
@@ -876,13 +876,13 @@
         <v>51</v>
       </c>
       <c r="C4" t="s" s="2">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s" s="2">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5">
@@ -893,7 +893,7 @@
         <v>53</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s" s="2">
         <v>42</v>
@@ -910,7 +910,7 @@
         <v>54</v>
       </c>
       <c r="C6" t="s" s="2">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s" s="2">
         <v>44</v>
@@ -927,7 +927,7 @@
         <v>55</v>
       </c>
       <c r="C7" t="s" s="2">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s" s="2">
         <v>46</v>

</xml_diff>